<commit_message>
Enhanced: daily exchange rates, column types, currency totals, error reporting
</commit_message>
<xml_diff>
--- a/test_exchange_rates.xlsx
+++ b/test_exchange_rates.xlsx
@@ -397,51 +397,154 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Currency Code</v>
+        <v>Date</v>
       </c>
       <c r="B1" t="str">
-        <v>Exchange Rate</v>
+        <v>Currency</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Rate</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
+        <v>2025-01-10</v>
+      </c>
+      <c r="B2" t="str">
+        <v>EUR</v>
+      </c>
+      <c r="C2">
+        <v>1.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EUR</v>
-      </c>
-      <c r="B3">
-        <v>1.08</v>
+        <v>2025-01-10</v>
+      </c>
+      <c r="B3" t="str">
+        <v>GBP</v>
+      </c>
+      <c r="C3">
+        <v>1.27</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GBP</v>
-      </c>
-      <c r="B4">
-        <v>1.27</v>
+        <v>2025-01-10</v>
+      </c>
+      <c r="B4" t="str">
+        <v>JPY</v>
+      </c>
+      <c r="C4">
+        <v>0.0067</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>2025-01-15</v>
+      </c>
+      <c r="B5" t="str">
+        <v>EUR</v>
+      </c>
+      <c r="C5">
+        <v>1.085</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2025-01-15</v>
+      </c>
+      <c r="B6" t="str">
+        <v>GBP</v>
+      </c>
+      <c r="C6">
+        <v>1.272</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2025-01-15</v>
+      </c>
+      <c r="B7" t="str">
         <v>JPY</v>
       </c>
-      <c r="B5">
-        <v>0.0067</v>
+      <c r="C7">
+        <v>0.0066</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2025-01-20</v>
+      </c>
+      <c r="B8" t="str">
+        <v>EUR</v>
+      </c>
+      <c r="C8">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2025-01-20</v>
+      </c>
+      <c r="B9" t="str">
+        <v>GBP</v>
+      </c>
+      <c r="C9">
+        <v>1.275</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2025-01-20</v>
+      </c>
+      <c r="B10" t="str">
+        <v>JPY</v>
+      </c>
+      <c r="C10">
+        <v>0.0065</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2025-01-25</v>
+      </c>
+      <c r="B11" t="str">
+        <v>EUR</v>
+      </c>
+      <c r="C11">
+        <v>1.087</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2025-01-25</v>
+      </c>
+      <c r="B12" t="str">
+        <v>GBP</v>
+      </c>
+      <c r="C12">
+        <v>1.268</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2025-01-25</v>
+      </c>
+      <c r="B13" t="str">
+        <v>JPY</v>
+      </c>
+      <c r="C13">
+        <v>0.0068</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>